<commit_message>
Adressen der PE-finanzierten Haeuser auf die eigene Gesellschaft korrigiert
Vier Zeilen standen auf der Mutter- oder Investorenadresse statt auf der des
Unternehmens selbst:
- Grant Thornton: Grant Thornton AG WPG, Duesseldorf statt Grant Thornton
  International, London. Land damit DE, Landzeile entfaellt.
- Unity: UNITY AG, Lindberghring 1, Bueren statt Deutsche Beteiligungs AG.
- interpath: Interpath Advisory, 10 Fleet Place, London statt Bridgepoint
  Group plc, 5 Marble Arch.
- wts global: dokumentiertes Postfach Rotterdam; eine Strassenanschrift
  veroeffentlicht WTS Global nicht.

Zusaetzlich eine Spalte mit dem jeweiligen Finanzinvestor. Zwei Haeuser der
Longlist tauchen dort selbst als Investor auf: Capza bei Epsa, H.I.G. Capital
bis Januar 2026 bei Interpath.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015H8odxAEQBbyd5de8uHVVB
</commit_message>
<xml_diff>
--- a/HQ_Adressen_Longlist.xlsx
+++ b/HQ_Adressen_Longlist.xlsx
@@ -10,7 +10,7 @@
     <sheet name="HQ-Adressen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HQ-Adressen'!$A$1:$E$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'HQ-Adressen'!$A$1:$F$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,14 +482,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -518,6 +519,11 @@
           <t>Adresse (Hauptsitz)</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Finanzinvestor / Eigentümer</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -547,6 +553,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F2" s="4" t="inlineStr"/>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -576,6 +583,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -605,6 +613,7 @@
 Vereinigtes Königreich</t>
         </is>
       </c>
+      <c r="F4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -634,6 +643,7 @@
 Vereinigtes Königreich</t>
         </is>
       </c>
+      <c r="F5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -663,6 +673,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -692,6 +703,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -721,6 +733,7 @@
 Vereinigtes Königreich</t>
         </is>
       </c>
+      <c r="F8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -750,6 +763,7 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -779,6 +793,7 @@
 Niederlande</t>
         </is>
       </c>
+      <c r="F10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -808,6 +823,7 @@
 Irland</t>
         </is>
       </c>
+      <c r="F11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -837,6 +853,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -865,6 +882,7 @@
 80538 München</t>
         </is>
       </c>
+      <c r="F13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -894,6 +912,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>CDPQ (La Caisse), PSP Investments, Investcorp + Gründer Jay Alix; CVC 2016 ausgestiegen</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -923,6 +946,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Madison Dearborn Partners (Mehrheit, seit 2016); HPS Investment Partners (Minderheit, 2021)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -952,6 +980,11 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Ardian (Wachstumskapital)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -981,6 +1014,11 @@
 Schweden</t>
         </is>
       </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Adelis Equity Partners (Minderheit)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1010,6 +1048,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Parthenon Capital (seit 06/2022, 15+ Zukäufe)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1039,6 +1082,11 @@
 Vereinigtes Königreich</t>
         </is>
       </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Tenzing (seit 2021)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1068,33 +1116,42 @@
 Frankreich</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>TowerBrook Capital Partners, Raise Investissement, Capza Expansion (Minderheiten)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Grant Thornton</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Prof. Dr. Heike Wieland-Blöse</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Europa</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>8 Finsbury Circus
-London EC2M 7EA
-Vereinigtes Königreich</t>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Johannstraße 39
+40476 Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Cinven - Mehrheit an Grant Thornton Deutschland, Partner-Zustimmung 10/2025, Closing Q1 2026</t>
         </is>
       </c>
     </row>
@@ -1121,9 +1178,14 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>5 Marble Arch
-London W1H 7EJ
+          <t>10 Fleet Place, 9th Floor
+London EC4M 7RB
 Vereinigtes Königreich</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Bridgepoint (seit 01/2026, ca. 800 Mio. GBP); vorher H.I.G. Capital</t>
         </is>
       </c>
     </row>
@@ -1155,6 +1217,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Konsortium unter Führung von Stone Point Capital und Further Global (2020); Permira mit Restbeteiligung</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1184,6 +1251,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Trivest Partners</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1213,6 +1285,11 @@
 USA</t>
         </is>
       </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>CVC Capital Partners (Mehrheit, 2019); LGT Capital Partners (Minderheit, 08/2025)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1237,8 +1314,13 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Untermainanlage 1
-60329 Frankfurt am Main</t>
+          <t>Lindberghring 1
+33142 Büren</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Deutsche Beteiligungs AG (Mehrheit seit 2024)</t>
         </is>
       </c>
     </row>
@@ -1265,9 +1347,14 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Registersitz Rotterdam - Strasse nicht belegt
-(operativ: Thomas-Wimmer-Ring 1, 80539 München)
+          <t>Postbus 19201
+3001 BE Rotterdam
 Niederlande</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>kein Finanzinvestor - partnergeführter Verbund</t>
         </is>
       </c>
     </row>
@@ -1299,6 +1386,7 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1327,6 +1415,7 @@
 80331 München</t>
         </is>
       </c>
+      <c r="F29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="46" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -1356,6 +1445,7 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F30" s="4" t="inlineStr"/>
     </row>
     <row r="31" ht="46" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -1385,6 +1475,7 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="46" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -1414,6 +1505,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="46" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -1443,6 +1535,7 @@
 Frankreich</t>
         </is>
       </c>
+      <c r="F33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="46" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -1472,6 +1565,7 @@
 Vereinigtes Königreich</t>
         </is>
       </c>
+      <c r="F34" s="4" t="inlineStr"/>
     </row>
     <row r="35" ht="46" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -1501,6 +1595,7 @@
 USA</t>
         </is>
       </c>
+      <c r="F35" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -1553,52 +1648,52 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Konzernebene statt Marke</t>
+          <t>Korrigiert: eigene Adresse statt Mutter oder Investor</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>FTI Andersch: FTI Consulting, Washington. Baker Tilly: Baker Tilly International, London. Grant Thornton: Grant Thornton International, London. KPMG: KPMG International, Amstelveen. Accenture: Accenture plc, Dublin. Oliver Wyman: Oliver Wyman LLC, New York (Konzern Marsh McLennan). Unity: Deutsche Beteiligungs AG, Frankfurt. interpath: Bridgepoint Group plc, London.</t>
+          <t>Grant Thornton: jetzt Grant Thornton AG Wirtschaftspruefungsgesellschaft, Duesseldorf - vorher irrtuemlich Grant Thornton International, London. Damit auch Land von GB auf DE, Landzeile entfaellt.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr"/>
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Unity: jetzt UNITY AG, Lindberghring 1, Bueren - vorher irrtuemlich die Deutsche Beteiligungs AG, Frankfurt.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>Unsichere Angaben</t>
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>interpath: jetzt Interpath Advisory, 10 Fleet Place, London - vorher irrtuemlich Bridgepoint Group plc, 5 Marble Arch.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>wts global: Fuer den Registersitz Rotterdam (Handelsregister Rotterdam, Nr. 50381903) ist nur ein Postfach dokumentiert, keine Strassenanschrift. Praktisch nutzbar ist die Muenchner Adresse der WTS Group AG.</t>
+          <t>wts global: jetzt das dokumentierte Postfach in Rotterdam. Eine Strassenanschrift veroeffentlicht WTS Global nicht; operativ nutzbar ist WTS Group AG, Thomas-Wimmer-Ring 1, 80539 Muenchen.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>Epsa: 19 rue Cognacq-Jay, 75007 Paris ist die Konzernanschrift. Das franzoesische Register fuehrt fuer die EPSA SA einen Sitz im 15. Arrondissement und fuer die EPSA Holding 65 rue d'Anjou, 75008 Paris.</t>
-        </is>
-      </c>
+      <c r="A50" s="9" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>interpath (Bridgepoint): 5 Marble Arch ist der eingetragene Sitz. 95 Wigmore Street taucht in Unterlagen als frueheres Korrespondenzbuero auf. Interpath selbst sitzt in London.</t>
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Noch offen: dieselbe Logik bei fuenf nicht-PE-Zeilen</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>Province: Die Firma nennt Las Vegas als Sitz, die dokumentierte Anschrift liegt aber in Henderson, Nevada.</t>
+          <t>Dort steht weiterhin die Konzern- statt der Markenadresse, weil die Marke keinen eigenen Hauptsitz hat: FTI Andersch (FTI Consulting, Washington), Baker Tilly (Baker Tilly International, London), KPMG (KPMG International, Amstelveen), Accenture (Accenture plc, Dublin), Oliver Wyman (Oliver Wyman LLC, New York). Sag Bescheid, wenn dort die deutsche Gesellschaft stehen soll - FTI-Andersch AG Frankfurt, Baker Tilly Deutschland, KPMG AG Berlin, Accenture Kronberg, Oliver Wyman GmbH Muenchen.</t>
         </is>
       </c>
     </row>
@@ -1608,36 +1703,98 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>Normalisiert gegenueber deiner Fassung</t>
+          <t>Unsichere Angaben</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Laendercodes auf ISO-3166-alpha-2 gebracht: GB statt UK (vier Zeilen). Ankura von EU auf US korrigiert. Sun Capital von UK/Europe auf US/Amerika. Region durchgaengig Europa statt Europe.</t>
+          <t>wts global: Fuer den Registersitz Rotterdam (Handelsregister Rotterdam, Nr. 50381903) ist nur ein Postfach dokumentiert, keine Strassenanschrift. Praktisch nutzbar ist die Muenchner Adresse der WTS Group AG.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="9" t="inlineStr"/>
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>Epsa: 19 rue Cognacq-Jay, 75007 Paris ist die Konzernanschrift. Das franzoesische Register fuehrt fuer die EPSA SA einen Sitz im 15. Arrondissement und fuer die EPSA Holding 65 rue d'Anjou, 75008 Paris.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>Einschraenkung</t>
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>interpath (Bridgepoint): 5 Marble Arch ist der eingetragene Sitz. 95 Wigmore Street taucht in Unterlagen als frueheres Korrespondenzbuero auf. Interpath selbst sitzt in London.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
+          <t>Province: Die Firma nennt Las Vegas als Sitz, die dokumentierte Anschrift liegt aber in Henderson, Nevada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Zur Investorenspalte</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>Zwei Haeuser deiner Longlist tauchen dort als Investor auf: Capza ist Minderheitsgesellschafter bei Epsa, H.I.G. Capital war bis Januar 2026 Eigentuemer von Interpath. Sie sind auf der Longlist also gleichzeitig Adressat und Gegenpartei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>Bei AlixPartners ist CVC seit 2016 ausgestiegen - dort halten CDPQ, PSP Investments und Investcorp neben dem Gruender Jay Alix. CVC ist heute bei Teneo investiert, nicht bei AlixPartners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>Normalisiert gegenueber deiner Fassung</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>Laendercodes auf ISO-3166-alpha-2 gebracht: GB statt UK (vier Zeilen). Ankura von EU auf US korrigiert. Sun Capital von UK/Europe auf US/Amerika. Region durchgaengig Europa statt Europe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Einschraenkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
           <t>Die Egress-Policy dieser Umgebung blockiert externe Seiten. Alle Adressen stammen aus Suchtreffern der jeweiligen Impressums-, Kontakt- und Registerquellen, keine wurde durch Seitenaufruf geprueft.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E35"/>
+  <autoFilter ref="A1:F35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>